<commit_message>
Kit Medicos: atendimento nunca condicionado a pagamento (planilha 14), numeros em formato pt-BR no cache das planilhas 12, 14 e 20, grupo Caixa explicado (41 prompts), poster do video escolhe quadro sem legenda
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-medicos/20-resumo-do-mes.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-medicos/20-resumo-do-mes.xlsx
@@ -923,23 +923,23 @@
       </c>
       <c r="B5" s="9" t="str">
         <f>IF(Q5="","",IF(Indicadores!B5="R$","R$ ","")&amp;FIXED(Q5,N5)&amp;IF(Indicadores!B5="%","%",IF(OR(Indicadores!B5="R$",Indicadores!B5="",Indicadores!B5="un"),""," "&amp;Indicadores!B5)))</f>
-        <v>R$ 49,651</v>
+        <v>R$ 49.651</v>
       </c>
       <c r="C5" s="9" t="str">
         <f>IF(R5="","",IF(Indicadores!B5="R$","R$ ","")&amp;FIXED(R5,N5)&amp;IF(Indicadores!B5="%","%",IF(OR(Indicadores!B5="R$",Indicadores!B5="",Indicadores!B5="un"),""," "&amp;Indicadores!B5)))</f>
-        <v>R$ 53,461</v>
+        <v>R$ 53.461</v>
       </c>
       <c r="D5" s="9" t="str">
         <f>IF(T5="","",IF(T5&gt;=0,"+","")&amp;IF(Indicadores!B5="%",FIXED(T5,1)&amp;" p.p.",FIXED(T5*100,1)&amp;"%"))</f>
-        <v>-7.1%</v>
+        <v>-7,1%</v>
       </c>
       <c r="E5" s="9" t="str">
         <f>IF(S5="","",IF(Indicadores!B5="R$","R$ ","")&amp;FIXED(S5,N5)&amp;IF(Indicadores!B5="%","%",IF(OR(Indicadores!B5="R$",Indicadores!B5="",Indicadores!B5="un"),""," "&amp;Indicadores!B5)))</f>
-        <v>R$ 46,000</v>
+        <v>R$ 46.000</v>
       </c>
       <c r="F5" s="9" t="str">
         <f>IF(U5="","",IF(U5&gt;=0,"+","")&amp;IF(Indicadores!B5="%",FIXED(U5,1)&amp;" p.p.",FIXED(U5*100,1)&amp;"%"))</f>
-        <v>+7.9%</v>
+        <v>+7,9%</v>
       </c>
       <c r="G5" s="9" t="str">
         <f>IF(OR(Q5="",S5=""),"",IF(Indicadores!E5="Não",IF(Q5&lt;=S5,"No alvo","Acima da meta"),IF(Q5&gt;=S5,"No alvo","Abaixo da meta")))</f>
@@ -989,23 +989,23 @@
       </c>
       <c r="B6" s="9" t="str">
         <f>IF(Q6="","",IF(Indicadores!B6="R$","R$ ","")&amp;FIXED(Q6,N6)&amp;IF(Indicadores!B6="%","%",IF(OR(Indicadores!B6="R$",Indicadores!B6="",Indicadores!B6="un"),""," "&amp;Indicadores!B6)))</f>
-        <v>R$ 42,583</v>
+        <v>R$ 42.583</v>
       </c>
       <c r="C6" s="9" t="str">
         <f>IF(R6="","",IF(Indicadores!B6="R$","R$ ","")&amp;FIXED(R6,N6)&amp;IF(Indicadores!B6="%","%",IF(OR(Indicadores!B6="R$",Indicadores!B6="",Indicadores!B6="un"),""," "&amp;Indicadores!B6)))</f>
-        <v>R$ 42,505</v>
+        <v>R$ 42.505</v>
       </c>
       <c r="D6" s="9" t="str">
         <f>IF(T6="","",IF(T6&gt;=0,"+","")&amp;IF(Indicadores!B6="%",FIXED(T6,1)&amp;" p.p.",FIXED(T6*100,1)&amp;"%"))</f>
-        <v>+0.2%</v>
+        <v>+0,2%</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>IF(S6="","",IF(Indicadores!B6="R$","R$ ","")&amp;FIXED(S6,N6)&amp;IF(Indicadores!B6="%","%",IF(OR(Indicadores!B6="R$",Indicadores!B6="",Indicadores!B6="un"),""," "&amp;Indicadores!B6)))</f>
-        <v>R$ 44,000</v>
+        <v>R$ 44.000</v>
       </c>
       <c r="F6" s="9" t="str">
         <f>IF(U6="","",IF(U6&gt;=0,"+","")&amp;IF(Indicadores!B6="%",FIXED(U6,1)&amp;" p.p.",FIXED(U6*100,1)&amp;"%"))</f>
-        <v>-3.2%</v>
+        <v>-3,2%</v>
       </c>
       <c r="G6" s="9" t="str">
         <f>IF(OR(Q6="",S6=""),"",IF(Indicadores!E6="Não",IF(Q6&lt;=S6,"No alvo","Acima da meta"),IF(Q6&gt;=S6,"No alvo","Abaixo da meta")))</f>
@@ -1055,23 +1055,23 @@
       </c>
       <c r="B7" s="9" t="str">
         <f>IF(Q7="","",IF(Indicadores!B7="R$","R$ ","")&amp;FIXED(Q7,N7)&amp;IF(Indicadores!B7="%","%",IF(OR(Indicadores!B7="R$",Indicadores!B7="",Indicadores!B7="un"),""," "&amp;Indicadores!B7)))</f>
-        <v>R$ 7,068</v>
+        <v>R$ 7.068</v>
       </c>
       <c r="C7" s="9" t="str">
         <f>IF(R7="","",IF(Indicadores!B7="R$","R$ ","")&amp;FIXED(R7,N7)&amp;IF(Indicadores!B7="%","%",IF(OR(Indicadores!B7="R$",Indicadores!B7="",Indicadores!B7="un"),""," "&amp;Indicadores!B7)))</f>
-        <v>R$ 10,956</v>
+        <v>R$ 10.956</v>
       </c>
       <c r="D7" s="9" t="str">
         <f>IF(T7="","",IF(T7&gt;=0,"+","")&amp;IF(Indicadores!B7="%",FIXED(T7,1)&amp;" p.p.",FIXED(T7*100,1)&amp;"%"))</f>
-        <v>-35.5%</v>
+        <v>-35,5%</v>
       </c>
       <c r="E7" s="9" t="str">
         <f>IF(S7="","",IF(Indicadores!B7="R$","R$ ","")&amp;FIXED(S7,N7)&amp;IF(Indicadores!B7="%","%",IF(OR(Indicadores!B7="R$",Indicadores!B7="",Indicadores!B7="un"),""," "&amp;Indicadores!B7)))</f>
-        <v>R$ 5,000</v>
+        <v>R$ 5.000</v>
       </c>
       <c r="F7" s="9" t="str">
         <f>IF(U7="","",IF(U7&gt;=0,"+","")&amp;IF(Indicadores!B7="%",FIXED(U7,1)&amp;" p.p.",FIXED(U7*100,1)&amp;"%"))</f>
-        <v>+41.4%</v>
+        <v>+41,4%</v>
       </c>
       <c r="G7" s="9" t="str">
         <f>IF(OR(Q7="",S7=""),"",IF(Indicadores!E7="Não",IF(Q7&lt;=S7,"No alvo","Acima da meta"),IF(Q7&gt;=S7,"No alvo","Abaixo da meta")))</f>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="U7" s="10">
         <f>IF(OR(Q7="",S7=""),"",IF(Indicadores!B7="%",Q7-S7,IF(S7=0,"",(Q7-S7)/ABS(S7))))</f>
-        <v>0.413576000000002</v>
+        <v>0.413576000000001</v>
       </c>
     </row>
     <row r="8">
@@ -1121,23 +1121,23 @@
       </c>
       <c r="B8" s="9" t="str">
         <f>IF(Q8="","",IF(Indicadores!B8="R$","R$ ","")&amp;FIXED(Q8,N8)&amp;IF(Indicadores!B8="%","%",IF(OR(Indicadores!B8="R$",Indicadores!B8="",Indicadores!B8="un"),""," "&amp;Indicadores!B8)))</f>
-        <v>14.2%</v>
+        <v>14,2%</v>
       </c>
       <c r="C8" s="9" t="str">
         <f>IF(R8="","",IF(Indicadores!B8="R$","R$ ","")&amp;FIXED(R8,N8)&amp;IF(Indicadores!B8="%","%",IF(OR(Indicadores!B8="R$",Indicadores!B8="",Indicadores!B8="un"),""," "&amp;Indicadores!B8)))</f>
-        <v>20.5%</v>
+        <v>20,5%</v>
       </c>
       <c r="D8" s="9" t="str">
         <f>IF(T8="","",IF(T8&gt;=0,"+","")&amp;IF(Indicadores!B8="%",FIXED(T8,1)&amp;" p.p.",FIXED(T8*100,1)&amp;"%"))</f>
-        <v>-6.3 p.p.</v>
+        <v>-6,3 p.p.</v>
       </c>
       <c r="E8" s="9" t="str">
         <f>IF(S8="","",IF(Indicadores!B8="R$","R$ ","")&amp;FIXED(S8,N8)&amp;IF(Indicadores!B8="%","%",IF(OR(Indicadores!B8="R$",Indicadores!B8="",Indicadores!B8="un"),""," "&amp;Indicadores!B8)))</f>
-        <v>12.0%</v>
+        <v>12,0%</v>
       </c>
       <c r="F8" s="9" t="str">
         <f>IF(U8="","",IF(U8&gt;=0,"+","")&amp;IF(Indicadores!B8="%",FIXED(U8,1)&amp;" p.p.",FIXED(U8*100,1)&amp;"%"))</f>
-        <v>+2.2 p.p.</v>
+        <v>+2,2 p.p.</v>
       </c>
       <c r="G8" s="9" t="str">
         <f>IF(OR(Q8="",S8=""),"",IF(Indicadores!E8="Não",IF(Q8&lt;=S8,"No alvo","Acima da meta"),IF(Q8&gt;=S8,"No alvo","Abaixo da meta")))</f>
@@ -1187,23 +1187,23 @@
       </c>
       <c r="B9" s="9" t="str">
         <f>IF(Q9="","",IF(Indicadores!B9="R$","R$ ","")&amp;FIXED(Q9,N9)&amp;IF(Indicadores!B9="%","%",IF(OR(Indicadores!B9="R$",Indicadores!B9="",Indicadores!B9="un"),""," "&amp;Indicadores!B9)))</f>
-        <v>70.4%</v>
+        <v>70,4%</v>
       </c>
       <c r="C9" s="9" t="str">
         <f>IF(R9="","",IF(Indicadores!B9="R$","R$ ","")&amp;FIXED(R9,N9)&amp;IF(Indicadores!B9="%","%",IF(OR(Indicadores!B9="R$",Indicadores!B9="",Indicadores!B9="un"),""," "&amp;Indicadores!B9)))</f>
-        <v>71.7%</v>
+        <v>71,7%</v>
       </c>
       <c r="D9" s="9" t="str">
         <f>IF(T9="","",IF(T9&gt;=0,"+","")&amp;IF(Indicadores!B9="%",FIXED(T9,1)&amp;" p.p.",FIXED(T9*100,1)&amp;"%"))</f>
-        <v>-1.3 p.p.</v>
+        <v>-1,3 p.p.</v>
       </c>
       <c r="E9" s="9" t="str">
         <f>IF(S9="","",IF(Indicadores!B9="R$","R$ ","")&amp;FIXED(S9,N9)&amp;IF(Indicadores!B9="%","%",IF(OR(Indicadores!B9="R$",Indicadores!B9="",Indicadores!B9="un"),""," "&amp;Indicadores!B9)))</f>
-        <v>75.0%</v>
+        <v>75,0%</v>
       </c>
       <c r="F9" s="9" t="str">
         <f>IF(U9="","",IF(U9&gt;=0,"+","")&amp;IF(Indicadores!B9="%",FIXED(U9,1)&amp;" p.p.",FIXED(U9*100,1)&amp;"%"))</f>
-        <v>-4.6 p.p.</v>
+        <v>-4,6 p.p.</v>
       </c>
       <c r="G9" s="9" t="str">
         <f>IF(OR(Q9="",S9=""),"",IF(Indicadores!E9="Não",IF(Q9&lt;=S9,"No alvo","Acima da meta"),IF(Q9&gt;=S9,"No alvo","Abaixo da meta")))</f>
@@ -1253,23 +1253,23 @@
       </c>
       <c r="B10" s="9" t="str">
         <f>IF(Q10="","",IF(Indicadores!B10="R$","R$ ","")&amp;FIXED(Q10,N10)&amp;IF(Indicadores!B10="%","%",IF(OR(Indicadores!B10="R$",Indicadores!B10="",Indicadores!B10="un"),""," "&amp;Indicadores!B10)))</f>
-        <v>8.4%</v>
+        <v>8,4%</v>
       </c>
       <c r="C10" s="9" t="str">
         <f>IF(R10="","",IF(Indicadores!B10="R$","R$ ","")&amp;FIXED(R10,N10)&amp;IF(Indicadores!B10="%","%",IF(OR(Indicadores!B10="R$",Indicadores!B10="",Indicadores!B10="un"),""," "&amp;Indicadores!B10)))</f>
-        <v>8.8%</v>
+        <v>8,8%</v>
       </c>
       <c r="D10" s="9" t="str">
         <f>IF(T10="","",IF(T10&gt;=0,"+","")&amp;IF(Indicadores!B10="%",FIXED(T10,1)&amp;" p.p.",FIXED(T10*100,1)&amp;"%"))</f>
-        <v>-0.4 p.p.</v>
+        <v>-0,4 p.p.</v>
       </c>
       <c r="E10" s="9" t="str">
         <f>IF(S10="","",IF(Indicadores!B10="R$","R$ ","")&amp;FIXED(S10,N10)&amp;IF(Indicadores!B10="%","%",IF(OR(Indicadores!B10="R$",Indicadores!B10="",Indicadores!B10="un"),""," "&amp;Indicadores!B10)))</f>
-        <v>6.0%</v>
+        <v>6,0%</v>
       </c>
       <c r="F10" s="9" t="str">
         <f>IF(U10="","",IF(U10&gt;=0,"+","")&amp;IF(Indicadores!B10="%",FIXED(U10,1)&amp;" p.p.",FIXED(U10*100,1)&amp;"%"))</f>
-        <v>+2.4 p.p.</v>
+        <v>+2,4 p.p.</v>
       </c>
       <c r="G10" s="9" t="str">
         <f>IF(OR(Q10="",S10=""),"",IF(Indicadores!E10="Não",IF(Q10&lt;=S10,"No alvo","Acima da meta"),IF(Q10&gt;=S10,"No alvo","Abaixo da meta")))</f>
@@ -1319,23 +1319,23 @@
       </c>
       <c r="B11" s="9" t="str">
         <f>IF(Q11="","",IF(Indicadores!B11="R$","R$ ","")&amp;FIXED(Q11,N11)&amp;IF(Indicadores!B11="%","%",IF(OR(Indicadores!B11="R$",Indicadores!B11="",Indicadores!B11="un"),""," "&amp;Indicadores!B11)))</f>
-        <v>118.3 h</v>
+        <v>118,3 h</v>
       </c>
       <c r="C11" s="9" t="str">
         <f>IF(R11="","",IF(Indicadores!B11="R$","R$ ","")&amp;FIXED(R11,N11)&amp;IF(Indicadores!B11="%","%",IF(OR(Indicadores!B11="R$",Indicadores!B11="",Indicadores!B11="un"),""," "&amp;Indicadores!B11)))</f>
-        <v>129.0 h</v>
+        <v>129,0 h</v>
       </c>
       <c r="D11" s="9" t="str">
         <f>IF(T11="","",IF(T11&gt;=0,"+","")&amp;IF(Indicadores!B11="%",FIXED(T11,1)&amp;" p.p.",FIXED(T11*100,1)&amp;"%"))</f>
-        <v>-8.3%</v>
+        <v>-8,3%</v>
       </c>
       <c r="E11" s="9" t="str">
         <f>IF(S11="","",IF(Indicadores!B11="R$","R$ ","")&amp;FIXED(S11,N11)&amp;IF(Indicadores!B11="%","%",IF(OR(Indicadores!B11="R$",Indicadores!B11="",Indicadores!B11="un"),""," "&amp;Indicadores!B11)))</f>
-        <v>140.0 h</v>
+        <v>140,0 h</v>
       </c>
       <c r="F11" s="9" t="str">
         <f>IF(U11="","",IF(U11&gt;=0,"+","")&amp;IF(Indicadores!B11="%",FIXED(U11,1)&amp;" p.p.",FIXED(U11*100,1)&amp;"%"))</f>
-        <v>-15.5%</v>
+        <v>-15,5%</v>
       </c>
       <c r="G11" s="9" t="str">
         <f>IF(OR(Q11="",S11=""),"",IF(Indicadores!E11="Não",IF(Q11&lt;=S11,"No alvo","Acima da meta"),IF(Q11&gt;=S11,"No alvo","Abaixo da meta")))</f>
@@ -1385,15 +1385,15 @@
       </c>
       <c r="B12" s="9" t="str">
         <f>IF(Q12="","",IF(Indicadores!B12="R$","R$ ","")&amp;FIXED(Q12,N12)&amp;IF(Indicadores!B12="%","%",IF(OR(Indicadores!B12="R$",Indicadores!B12="",Indicadores!B12="un"),""," "&amp;Indicadores!B12)))</f>
-        <v>R$ 12,077</v>
+        <v>R$ 12.077</v>
       </c>
       <c r="C12" s="9" t="str">
         <f>IF(R12="","",IF(Indicadores!B12="R$","R$ ","")&amp;FIXED(R12,N12)&amp;IF(Indicadores!B12="%","%",IF(OR(Indicadores!B12="R$",Indicadores!B12="",Indicadores!B12="un"),""," "&amp;Indicadores!B12)))</f>
-        <v>R$ 13,553</v>
+        <v>R$ 13.553</v>
       </c>
       <c r="D12" s="9" t="str">
         <f>IF(T12="","",IF(T12&gt;=0,"+","")&amp;IF(Indicadores!B12="%",FIXED(T12,1)&amp;" p.p.",FIXED(T12*100,1)&amp;"%"))</f>
-        <v>-10.9%</v>
+        <v>-10,9%</v>
       </c>
       <c r="E12" s="9">
         <f>IF(S12="","",IF(Indicadores!B12="R$","R$ ","")&amp;FIXED(S12,N12)&amp;IF(Indicadores!B12="%","%",IF(OR(Indicadores!B12="R$",Indicadores!B12="",Indicadores!B12="un"),""," "&amp;Indicadores!B12)))</f>
@@ -1451,23 +1451,23 @@
       </c>
       <c r="B13" s="9" t="str">
         <f>IF(Q13="","",IF(Indicadores!B13="R$","R$ ","")&amp;FIXED(Q13,N13)&amp;IF(Indicadores!B13="%","%",IF(OR(Indicadores!B13="R$",Indicadores!B13="",Indicadores!B13="un"),""," "&amp;Indicadores!B13)))</f>
-        <v>5.6%</v>
+        <v>5,6%</v>
       </c>
       <c r="C13" s="9" t="str">
         <f>IF(R13="","",IF(Indicadores!B13="R$","R$ ","")&amp;FIXED(R13,N13)&amp;IF(Indicadores!B13="%","%",IF(OR(Indicadores!B13="R$",Indicadores!B13="",Indicadores!B13="un"),""," "&amp;Indicadores!B13)))</f>
-        <v>4.3%</v>
+        <v>4,3%</v>
       </c>
       <c r="D13" s="9" t="str">
         <f>IF(T13="","",IF(T13&gt;=0,"+","")&amp;IF(Indicadores!B13="%",FIXED(T13,1)&amp;" p.p.",FIXED(T13*100,1)&amp;"%"))</f>
-        <v>+1.3 p.p.</v>
+        <v>+1,3 p.p.</v>
       </c>
       <c r="E13" s="9" t="str">
         <f>IF(S13="","",IF(Indicadores!B13="R$","R$ ","")&amp;FIXED(S13,N13)&amp;IF(Indicadores!B13="%","%",IF(OR(Indicadores!B13="R$",Indicadores!B13="",Indicadores!B13="un"),""," "&amp;Indicadores!B13)))</f>
-        <v>4.0%</v>
+        <v>4,0%</v>
       </c>
       <c r="F13" s="9" t="str">
         <f>IF(U13="","",IF(U13&gt;=0,"+","")&amp;IF(Indicadores!B13="%",FIXED(U13,1)&amp;" p.p.",FIXED(U13*100,1)&amp;"%"))</f>
-        <v>+1.6 p.p.</v>
+        <v>+1,6 p.p.</v>
       </c>
       <c r="G13" s="9" t="str">
         <f>IF(OR(Q13="",S13=""),"",IF(Indicadores!E13="Não",IF(Q13&lt;=S13,"No alvo","Acima da meta"),IF(Q13&gt;=S13,"No alvo","Abaixo da meta")))</f>
@@ -1517,23 +1517,23 @@
       </c>
       <c r="B14" s="9" t="str">
         <f>IF(Q14="","",IF(Indicadores!B14="R$","R$ ","")&amp;FIXED(Q14,N14)&amp;IF(Indicadores!B14="%","%",IF(OR(Indicadores!B14="R$",Indicadores!B14="",Indicadores!B14="un"),""," "&amp;Indicadores!B14)))</f>
-        <v>R$ 4,005</v>
+        <v>R$ 4.005</v>
       </c>
       <c r="C14" s="9" t="str">
         <f>IF(R14="","",IF(Indicadores!B14="R$","R$ ","")&amp;FIXED(R14,N14)&amp;IF(Indicadores!B14="%","%",IF(OR(Indicadores!B14="R$",Indicadores!B14="",Indicadores!B14="un"),""," "&amp;Indicadores!B14)))</f>
-        <v>R$ 3,290</v>
+        <v>R$ 3.290</v>
       </c>
       <c r="D14" s="9" t="str">
         <f>IF(T14="","",IF(T14&gt;=0,"+","")&amp;IF(Indicadores!B14="%",FIXED(T14,1)&amp;" p.p.",FIXED(T14*100,1)&amp;"%"))</f>
-        <v>+21.7%</v>
+        <v>+21,7%</v>
       </c>
       <c r="E14" s="9" t="str">
         <f>IF(S14="","",IF(Indicadores!B14="R$","R$ ","")&amp;FIXED(S14,N14)&amp;IF(Indicadores!B14="%","%",IF(OR(Indicadores!B14="R$",Indicadores!B14="",Indicadores!B14="un"),""," "&amp;Indicadores!B14)))</f>
-        <v>R$ 4,000</v>
+        <v>R$ 4.000</v>
       </c>
       <c r="F14" s="9" t="str">
         <f>IF(U14="","",IF(U14&gt;=0,"+","")&amp;IF(Indicadores!B14="%",FIXED(U14,1)&amp;" p.p.",FIXED(U14*100,1)&amp;"%"))</f>
-        <v>+0.1%</v>
+        <v>+0,1%</v>
       </c>
       <c r="G14" s="9" t="str">
         <f>IF(OR(Q14="",S14=""),"",IF(Indicadores!E14="Não",IF(Q14&lt;=S14,"No alvo","Acima da meta"),IF(Q14&gt;=S14,"No alvo","Abaixo da meta")))</f>
@@ -1583,23 +1583,23 @@
       </c>
       <c r="B15" s="9" t="str">
         <f>IF(Q15="","",IF(Indicadores!B15="R$","R$ ","")&amp;FIXED(Q15,N15)&amp;IF(Indicadores!B15="%","%",IF(OR(Indicadores!B15="R$",Indicadores!B15="",Indicadores!B15="un"),""," "&amp;Indicadores!B15)))</f>
-        <v>10.5%</v>
+        <v>10,5%</v>
       </c>
       <c r="C15" s="9" t="str">
         <f>IF(R15="","",IF(Indicadores!B15="R$","R$ ","")&amp;FIXED(R15,N15)&amp;IF(Indicadores!B15="%","%",IF(OR(Indicadores!B15="R$",Indicadores!B15="",Indicadores!B15="un"),""," "&amp;Indicadores!B15)))</f>
-        <v>10.0%</v>
+        <v>10,0%</v>
       </c>
       <c r="D15" s="9" t="str">
         <f>IF(T15="","",IF(T15&gt;=0,"+","")&amp;IF(Indicadores!B15="%",FIXED(T15,1)&amp;" p.p.",FIXED(T15*100,1)&amp;"%"))</f>
-        <v>+0.5 p.p.</v>
+        <v>+0,5 p.p.</v>
       </c>
       <c r="E15" s="9" t="str">
         <f>IF(S15="","",IF(Indicadores!B15="R$","R$ ","")&amp;FIXED(S15,N15)&amp;IF(Indicadores!B15="%","%",IF(OR(Indicadores!B15="R$",Indicadores!B15="",Indicadores!B15="un"),""," "&amp;Indicadores!B15)))</f>
-        <v>8.0%</v>
+        <v>8,0%</v>
       </c>
       <c r="F15" s="9" t="str">
         <f>IF(U15="","",IF(U15&gt;=0,"+","")&amp;IF(Indicadores!B15="%",FIXED(U15,1)&amp;" p.p.",FIXED(U15*100,1)&amp;"%"))</f>
-        <v>+2.5 p.p.</v>
+        <v>+2,5 p.p.</v>
       </c>
       <c r="G15" s="9" t="str">
         <f>IF(OR(Q15="",S15=""),"",IF(Indicadores!E15="Não",IF(Q15&lt;=S15,"No alvo","Acima da meta"),IF(Q15&gt;=S15,"No alvo","Abaixo da meta")))</f>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B16" s="9" t="str">
         <f>IF(Q16="","",IF(Indicadores!B16="R$","R$ ","")&amp;FIXED(Q16,N16)&amp;IF(Indicadores!B16="%","%",IF(OR(Indicadores!B16="R$",Indicadores!B16="",Indicadores!B16="un"),""," "&amp;Indicadores!B16)))</f>
-        <v>R$ 2,700</v>
+        <v>R$ 2.700</v>
       </c>
       <c r="C16" s="9" t="str">
         <f>IF(R16="","",IF(Indicadores!B16="R$","R$ ","")&amp;FIXED(R16,N16)&amp;IF(Indicadores!B16="%","%",IF(OR(Indicadores!B16="R$",Indicadores!B16="",Indicadores!B16="un"),""," "&amp;Indicadores!B16)))</f>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="D16" s="9" t="str">
         <f>IF(T16="","",IF(T16&gt;=0,"+","")&amp;IF(Indicadores!B16="%",FIXED(T16,1)&amp;" p.p.",FIXED(T16*100,1)&amp;"%"))</f>
-        <v>+225.3%</v>
+        <v>+225,3%</v>
       </c>
       <c r="E16" s="9">
         <f>IF(S16="","",IF(Indicadores!B16="R$","R$ ","")&amp;FIXED(S16,N16)&amp;IF(Indicadores!B16="%","%",IF(OR(Indicadores!B16="R$",Indicadores!B16="",Indicadores!B16="un"),""," "&amp;Indicadores!B16)))</f>
@@ -1792,73 +1792,73 @@
     <row r="8">
       <c r="A8" s="17" t="str">
         <f>IF(OR(Painel!A5="",Painel!Q5=""),"","• "&amp;Painel!A5&amp;": "&amp;Painel!B5&amp;IF(Painel!T5&lt;&gt;"",IF(Painel!T5=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D5&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R5&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S5&lt;&gt;"","; meta "&amp;Painel!E5&amp;", "&amp;LOWER(Painel!G5),"")&amp;".")</f>
-        <v>• Entrou no mês (recebimentos): R$ 49,651 (-7.1% em relação a Julho); meta R$ 46,000, no alvo.</v>
+        <v>• Entrou no mês (recebimentos): R$ 49.651 (-7,1% em relação a Julho); meta R$ 46.000, no alvo.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="str">
         <f>IF(OR(Painel!A6="",Painel!Q6=""),"","• "&amp;Painel!A6&amp;": "&amp;Painel!B6&amp;IF(Painel!T6&lt;&gt;"",IF(Painel!T6=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D6&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R6&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S6&lt;&gt;"","; meta "&amp;Painel!E6&amp;", "&amp;LOWER(Painel!G6),"")&amp;".")</f>
-        <v>• Saídas do mês (custos, variáveis, pró-labore, provisões e impostos): R$ 42,583 (+0.2% em relação a Julho); meta R$ 44,000, no alvo.</v>
+        <v>• Saídas do mês (custos, variáveis, pró-labore, provisões e impostos): R$ 42.583 (+0,2% em relação a Julho); meta R$ 44.000, no alvo.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="str">
         <f>IF(OR(Painel!A7="",Painel!Q7=""),"","• "&amp;Painel!A7&amp;": "&amp;Painel!B7&amp;IF(Painel!T7&lt;&gt;"",IF(Painel!T7=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D7&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R7&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S7&lt;&gt;"","; meta "&amp;Painel!E7&amp;", "&amp;LOWER(Painel!G7),"")&amp;".")</f>
-        <v>• Resultado do mês: R$ 7,068 (-35.5% em relação a Julho); meta R$ 5,000, no alvo.</v>
+        <v>• Resultado do mês: R$ 7.068 (-35,5% em relação a Julho); meta R$ 5.000, no alvo.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="str">
         <f>IF(OR(Painel!A8="",Painel!Q8=""),"","• "&amp;Painel!A8&amp;": "&amp;Painel!B8&amp;IF(Painel!T8&lt;&gt;"",IF(Painel!T8=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D8&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R8&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S8&lt;&gt;"","; meta "&amp;Painel!E8&amp;", "&amp;LOWER(Painel!G8),"")&amp;".")</f>
-        <v>• Margem do mês: 14.2% (-6.3 p.p. em relação a Julho); meta 12.0%, no alvo.</v>
+        <v>• Margem do mês: 14,2% (-6,3 p.p. em relação a Julho); meta 12,0%, no alvo.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="str">
         <f>IF(OR(Painel!A9="",Painel!Q9=""),"","• "&amp;Painel!A9&amp;": "&amp;Painel!B9&amp;IF(Painel!T9&lt;&gt;"",IF(Painel!T9=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D9&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R9&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S9&lt;&gt;"","; meta "&amp;Painel!E9&amp;", "&amp;LOWER(Painel!G9),"")&amp;".")</f>
-        <v>• Ocupação da agenda: 70.4% (-1.3 p.p. em relação a Julho); meta 75.0%, abaixo da meta.</v>
+        <v>• Ocupação da agenda: 70,4% (-1,3 p.p. em relação a Julho); meta 75,0%, abaixo da meta.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="str">
         <f>IF(OR(Painel!A10="",Painel!Q10=""),"","• "&amp;Painel!A10&amp;": "&amp;Painel!B10&amp;IF(Painel!T10&lt;&gt;"",IF(Painel!T10=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D10&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R10&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S10&lt;&gt;"","; meta "&amp;Painel!E10&amp;", "&amp;LOWER(Painel!G10),"")&amp;".")</f>
-        <v>• Taxa de falta: 8.4% (-0.4 p.p. em relação a Julho); meta 6.0%, acima da meta.</v>
+        <v>• Taxa de falta: 8,4% (-0,4 p.p. em relação a Julho); meta 6,0%, acima da meta.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="str">
         <f>IF(OR(Painel!A11="",Painel!Q11=""),"","• "&amp;Painel!A11&amp;": "&amp;Painel!B11&amp;IF(Painel!T11&lt;&gt;"",IF(Painel!T11=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D11&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R11&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S11&lt;&gt;"","; meta "&amp;Painel!E11&amp;", "&amp;LOWER(Painel!G11),"")&amp;".")</f>
-        <v>• Horas atendidas no mês: 118.3 h (-8.3% em relação a Julho); meta 140.0 h, abaixo da meta.</v>
+        <v>• Horas atendidas no mês: 118,3 h (-8,3% em relação a Julho); meta 140,0 h, abaixo da meta.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="str">
         <f>IF(OR(Painel!A12="",Painel!Q12=""),"","• "&amp;Painel!A12&amp;": "&amp;Painel!B12&amp;IF(Painel!T12&lt;&gt;"",IF(Painel!T12=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D12&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R12&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S12&lt;&gt;"","; meta "&amp;Painel!E12&amp;", "&amp;LOWER(Painel!G12),"")&amp;".")</f>
-        <v>• Convênio a receber (lotes enviados): R$ 12,077 (-10.9% em relação a Julho).</v>
+        <v>• Convênio a receber (lotes enviados): R$ 12.077 (-10,9% em relação a Julho).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="str">
         <f>IF(OR(Painel!A13="",Painel!Q13=""),"","• "&amp;Painel!A13&amp;": "&amp;Painel!B13&amp;IF(Painel!T13&lt;&gt;"",IF(Painel!T13=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D13&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R13&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S13&lt;&gt;"","; meta "&amp;Painel!E13&amp;", "&amp;LOWER(Painel!G13),"")&amp;".")</f>
-        <v>• Glosa dos lotes pagos no mês: 5.6% (+1.3 p.p. em relação a Julho); meta 4.0%, acima da meta.</v>
+        <v>• Glosa dos lotes pagos no mês: 5,6% (+1,3 p.p. em relação a Julho); meta 4,0%, acima da meta.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="str">
         <f>IF(OR(Painel!A14="",Painel!Q14=""),"","• "&amp;Painel!A14&amp;": "&amp;Painel!B14&amp;IF(Painel!T14&lt;&gt;"",IF(Painel!T14=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D14&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R14&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S14&lt;&gt;"","; meta "&amp;Painel!E14&amp;", "&amp;LOWER(Painel!G14),"")&amp;".")</f>
-        <v>• Vencido (parcelas a prazo): R$ 4,005 (+21.7% em relação a Julho); meta R$ 4,000, acima da meta.</v>
+        <v>• Vencido (parcelas a prazo): R$ 4.005 (+21,7% em relação a Julho); meta R$ 4.000, acima da meta.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="str">
         <f>IF(OR(Painel!A15="",Painel!Q15=""),"","• "&amp;Painel!A15&amp;": "&amp;Painel!B15&amp;IF(Painel!T15&lt;&gt;"",IF(Painel!T15=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D15&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R15&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S15&lt;&gt;"","; meta "&amp;Painel!E15&amp;", "&amp;LOWER(Painel!G15),"")&amp;".")</f>
-        <v>• Inadimplência a prazo (vencido ÷ (pago + vencido)): 10.5% (+0.5 p.p. em relação a Julho); meta 8.0%, acima da meta.</v>
+        <v>• Inadimplência a prazo (vencido ÷ (pago + vencido)): 10,5% (+0,5 p.p. em relação a Julho); meta 8,0%, acima da meta.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="str">
         <f>IF(OR(Painel!A16="",Painel!Q16=""),"","• "&amp;Painel!A16&amp;": "&amp;Painel!B16&amp;IF(Painel!T16&lt;&gt;"",IF(Painel!T16=0," (igual a "&amp;Config!$B$8&amp;")"," ("&amp;Painel!D16&amp;" em relação a "&amp;Config!$B$8&amp;")"),IF(Painel!R16&lt;&gt;""," (igual a "&amp;Config!$B$8&amp;")",""))&amp;IF(Painel!S16&lt;&gt;"","; meta "&amp;Painel!E16&amp;", "&amp;LOWER(Painel!G16),"")&amp;".")</f>
-        <v>• Orçamentos em aberto (valor): R$ 2,700 (+225.3% em relação a Julho).</v>
+        <v>• Orçamentos em aberto (valor): R$ 2.700 (+225,3% em relação a Julho).</v>
       </c>
     </row>
     <row r="20"/>
@@ -1872,19 +1872,19 @@
     <row r="22">
       <c r="A22" s="17" t="str">
         <f>IF(COUNT(Painel!$P$5:$P$16)=0,"• Melhora e piora: preencha o mês anterior para comparar.",IF(MAX(Painel!$P$5:$P$16)&lt;=0,"• Nenhum indicador melhorou contra "&amp;Config!$B$8&amp;".","• Maior melhora contra "&amp;Config!$B$8&amp;": "&amp;INDEX(Painel!$A$5:$A$16,MATCH(MAX(Painel!$P$5:$P$16),Painel!$P$5:$P$16,0))&amp;" ("&amp;INDEX(Painel!$D$5:$D$16,MATCH(MAX(Painel!$P$5:$P$16),Painel!$P$5:$P$16,0))&amp;")."))</f>
-        <v>• Maior melhora contra Julho: Orçamentos em aberto (valor) (+225.3%).</v>
+        <v>• Maior melhora contra Julho: Orçamentos em aberto (valor) (+225,3%).</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="str">
         <f>IF(COUNT(Painel!$P$5:$P$16)=0,"",IF(MIN(Painel!$P$5:$P$16)&gt;=0,"• Nenhum indicador piorou contra "&amp;Config!$B$8&amp;".","• Maior piora contra "&amp;Config!$B$8&amp;": "&amp;INDEX(Painel!$A$5:$A$16,MATCH(MIN(Painel!$P$5:$P$16),Painel!$P$5:$P$16,0))&amp;" ("&amp;INDEX(Painel!$D$5:$D$16,MATCH(MIN(Painel!$P$5:$P$16),Painel!$P$5:$P$16,0))&amp;")."))</f>
-        <v>• Maior piora contra Julho: Margem do mês (-6.3 p.p.).</v>
+        <v>• Maior piora contra Julho: Margem do mês (-6,3 p.p.).</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="str">
         <f>IF(COUNT(Painel!$O$5:$O$16)=0,"• Nenhum indicador fora da meta.","• Mais longe da meta: "&amp;INDEX(Painel!$A$5:$A$16,MATCH(MAX(Painel!$O$5:$O$16),Painel!$O$5:$O$16,0))&amp;" ("&amp;INDEX(Painel!$F$5:$F$16,MATCH(MAX(Painel!$O$5:$O$16),Painel!$O$5:$O$16,0))&amp;" da meta, "&amp;LOWER(INDEX(Painel!$G$5:$G$16,MATCH(MAX(Painel!$O$5:$O$16),Painel!$O$5:$O$16,0)))&amp;").")</f>
-        <v>• Mais longe da meta: Ocupação da agenda (-4.6 p.p. da meta, abaixo da meta).</v>
+        <v>• Mais longe da meta: Ocupação da agenda (-4,6 p.p. da meta, abaixo da meta).</v>
       </c>
     </row>
     <row r="25">
@@ -1906,22 +1906,22 @@
         <f>A4&amp;CHAR(10)&amp;CHAR(10)&amp;"Indicadores do mês:"&amp;CHAR(10)&amp;IF(A8="","",A8&amp;CHAR(10)) &amp; IF(A9="","",A9&amp;CHAR(10)) &amp; IF(A10="","",A10&amp;CHAR(10)) &amp; IF(A11="","",A11&amp;CHAR(10)) &amp; IF(A12="","",A12&amp;CHAR(10)) &amp; IF(A13="","",A13&amp;CHAR(10)) &amp; IF(A14="","",A14&amp;CHAR(10)) &amp; IF(A15="","",A15&amp;CHAR(10)) &amp; IF(A16="","",A16&amp;CHAR(10)) &amp; IF(A17="","",A17&amp;CHAR(10)) &amp; IF(A18="","",A18&amp;CHAR(10)) &amp; IF(A19="","",A19&amp;CHAR(10))&amp;CHAR(10)&amp;"Destaques:"&amp;CHAR(10)&amp;IF(A22="","",A22&amp;CHAR(10)) &amp; IF(A23="","",A23&amp;CHAR(10)) &amp; IF(A24="","",A24&amp;CHAR(10)) &amp; IF(A25="","",A25&amp;CHAR(10))&amp;IF(A6="","",CHAR(10)&amp;"Observações da clínica: "&amp;A6)</f>
         <v>Resumo de Agosto de 2026 · Clínica Vida Plena (exemplo fictício)
 Indicadores do mês:
-• Entrou no mês (recebimentos): R$ 49,651 (-7.1% em relação a Julho); meta R$ 46,000, no alvo.
-• Saídas do mês (custos, variáveis, pró-labore, provisões e impostos): R$ 42,583 (+0.2% em relação a Julho); meta R$ 44,000, no alvo.
-• Resultado do mês: R$ 7,068 (-35.5% em relação a Julho); meta R$ 5,000, no alvo.
-• Margem do mês: 14.2% (-6.3 p.p. em relação a Julho); meta 12.0%, no alvo.
-• Ocupação da agenda: 70.4% (-1.3 p.p. em relação a Julho); meta 75.0%, abaixo da meta.
-• Taxa de falta: 8.4% (-0.4 p.p. em relação a Julho); meta 6.0%, acima da meta.
-• Horas atendidas no mês: 118.3 h (-8.3% em relação a Julho); meta 140.0 h, abaixo da meta.
-• Convênio a receber (lotes enviados): R$ 12,077 (-10.9% em relação a Julho).
-• Glosa dos lotes pagos no mês: 5.6% (+1.3 p.p. em relação a Julho); meta 4.0%, acima da meta.
-• Vencido (parcelas a prazo): R$ 4,005 (+21.7% em relação a Julho); meta R$ 4,000, acima da meta.
-• Inadimplência a prazo (vencido ÷ (pago + vencido)): 10.5% (+0.5 p.p. em relação a Julho); meta 8.0%, acima da meta.
-• Orçamentos em aberto (valor): R$ 2,700 (+225.3% em relação a Julho).
+• Entrou no mês (recebimentos): R$ 49.651 (-7,1% em relação a Julho); meta R$ 46.000, no alvo.
+• Saídas do mês (custos, variáveis, pró-labore, provisões e impostos): R$ 42.583 (+0,2% em relação a Julho); meta R$ 44.000, no alvo.
+• Resultado do mês: R$ 7.068 (-35,5% em relação a Julho); meta R$ 5.000, no alvo.
+• Margem do mês: 14,2% (-6,3 p.p. em relação a Julho); meta 12,0%, no alvo.
+• Ocupação da agenda: 70,4% (-1,3 p.p. em relação a Julho); meta 75,0%, abaixo da meta.
+• Taxa de falta: 8,4% (-0,4 p.p. em relação a Julho); meta 6,0%, acima da meta.
+• Horas atendidas no mês: 118,3 h (-8,3% em relação a Julho); meta 140,0 h, abaixo da meta.
+• Convênio a receber (lotes enviados): R$ 12.077 (-10,9% em relação a Julho).
+• Glosa dos lotes pagos no mês: 5,6% (+1,3 p.p. em relação a Julho); meta 4,0%, acima da meta.
+• Vencido (parcelas a prazo): R$ 4.005 (+21,7% em relação a Julho); meta R$ 4.000, acima da meta.
+• Inadimplência a prazo (vencido ÷ (pago + vencido)): 10,5% (+0,5 p.p. em relação a Julho); meta 8,0%, acima da meta.
+• Orçamentos em aberto (valor): R$ 2.700 (+225,3% em relação a Julho).
 Destaques:
-• Maior melhora contra Julho: Orçamentos em aberto (valor) (+225.3%).
-• Maior piora contra Julho: Margem do mês (-6.3 p.p.).
-• Mais longe da meta: Ocupação da agenda (-4.6 p.p. da meta, abaixo da meta).
+• Maior melhora contra Julho: Orçamentos em aberto (valor) (+225,3%).
+• Maior piora contra Julho: Margem do mês (-6,3 p.p.).
+• Mais longe da meta: Ocupação da agenda (-4,6 p.p. da meta, abaixo da meta).
 • Indicadores no alvo: 4 de 10 com meta.
 Observações da clínica: Agosto fechou com a agenda da Dra. Renata mais cheia (dois turnos por semana desde julho) e o lote de junho da Saúde Total pago com glosa, parte dela em recurso; o lote de junho da Vida Care tinha previsão para 04/09 e ainda estava dentro do prazo no fechamento de agosto — em setembro venceu e entrou na cobrança ao convênio; as faltas de segunda de manhã continuam acima da média e a recepção começou a confirmação de véspera por mensagem.</v>
       </c>

</xml_diff>